<commit_message>
🎨 Update: Apply sidebar layout and Figurella styling
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Leads" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Consultation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Opportunity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Attendance" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,13 +420,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -437,322 +444,373 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>gfd</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>fgd</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>fgd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>fgd</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gsgssg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Lead Name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Lead Date</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Lead Source</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dfg</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>gfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Shehsh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-06-19</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Dgsgsg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dhsg</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-06-26</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Shsh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Consultation Name</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Consultation Outcome</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Consultation Source</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>fgd</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>gf</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fdg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Opportunity Name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Opportunity Provider</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Opportunity Description</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>fgd</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>fgd</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>gfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>fgdgfd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>gfd</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>gfd</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Attendances Done</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>No Show</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-06-13 23:21:31</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>h</t>
+      <c r="A2" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-06-13 23:22:08</t>
-        </is>
+      <c r="A3" s="1" t="n">
+        <v>45822</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-06-13 23:25:39</t>
-        </is>
+      <c r="A4" s="1" t="n">
+        <v>45822</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-06-13 23:32:28</t>
-        </is>
+      <c r="A5" s="1" t="n">
+        <v>45822</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>v</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>vc</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>kj</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>jk</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🚀 Update: Mobile sidebar toggle and Figurella styling
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -734,7 +734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -814,6 +814,21 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>